<commit_message>
Styles part didn't have correct count for number format
The count was negative, because not all ids reserved for the predefined
number formats are used. There is only ~29 predefined formats, but it
used 164. The final count was therefore negative. The XSD says count is
unsigned int and negative numbers are invalid per XSD.

The detection whether the format is predefined or not was also improved.
There could be (in theory) custom number formats in space allocated
for the predefined formats.

The test resource had pretty wonky styles part, the input didn't have
correctly connected cellXfs to cell styles. The input was having custom
number formats at (166, 200). The output was updated per new writer.
The custom number formats are now written into the first available slots
(164,165,166).

Fixes AddCustomNumberFormatsToFileWithNonSequentialNumberFormatIds
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Other/NumberFormats/NonSequentialNumberFormatsIds-Input.xlsx
+++ b/ClosedXML.Tests/Resource/Other/NumberFormats/NonSequentialNumberFormatsIds-Input.xlsx
@@ -90,8 +90,8 @@
   </x:cellStyleXfs>
   <x:cellXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <x:xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>